<commit_message>
3110 with aadhar changes
</commit_message>
<xml_diff>
--- a/input/Contractor.xlsx
+++ b/input/Contractor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Talntx_MobileAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35ECB3A-8FD6-4ABA-8870-EE4F7C706A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9BBAA2-15BA-4E3E-B288-E8AA646697C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="15375" windowHeight="7785" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
   </bookViews>
   <sheets>
     <sheet name="CEWithAadhar" sheetId="1" r:id="rId1"/>

</xml_diff>